<commit_message>
Add experiment setup with stimuli loading and jsPsych integration
</commit_message>
<xml_diff>
--- a/stimuli.xlsx
+++ b/stimuli.xlsx
@@ -137,7 +137,7 @@
     <t>Image1</t>
   </si>
   <si>
-    <t>Clear</t>
+    <t>Safe</t>
   </si>
   <si>
     <t xml:space="preserve">See comments indicated by red triangles for more information on the columns.</t>
@@ -215,7 +215,7 @@
     <t>Image25</t>
   </si>
   <si>
-    <t>Search</t>
+    <t>Danger</t>
   </si>
   <si>
     <t>Image26</t>
@@ -744,7 +744,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Stephanie Merritt" id="{023F073C-A82F-2175-A266-BCA5468DB114}"/>
+  <person displayName="Stephanie Merritt" id="{6CBFD0F5-E47F-8D54-1A2F-22C85849A140}"/>
 </personList>
 </file>
 
@@ -1228,20 +1228,20 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" personId="{023F073C-A82F-2175-A266-BCA5468DB114}" id="{61DA1E78-F749-1C58-6BBD-88174388418E}" done="0">
+  <threadedComment ref="A1" personId="{6CBFD0F5-E47F-8D54-1A2F-22C85849A140}" id="{61DA1E78-F749-1C58-6BBD-88174388418E}" done="0">
     <text xml:space="preserve">Slide names correspond to the images stored in the repository.
 </text>
   </threadedComment>
-  <threadedComment ref="B1" personId="{023F073C-A82F-2175-A266-BCA5468DB114}" id="{02C85690-7339-042A-0A1F-0D5D5E549D1A}" done="0">
+  <threadedComment ref="B1" personId="{6CBFD0F5-E47F-8D54-1A2F-22C85849A140}" id="{02C85690-7339-042A-0A1F-0D5D5E549D1A}" done="0">
     <text xml:space="preserve">Number of item in the suitcase
 </text>
   </threadedComment>
-  <threadedComment ref="C1" personId="{023F073C-A82F-2175-A266-BCA5468DB114}" id="{5AC044C2-1238-88F5-9AA8-317088AE8511}" done="0">
+  <threadedComment ref="C1" personId="{6CBFD0F5-E47F-8D54-1A2F-22C85849A140}" id="{5AC044C2-1238-88F5-9AA8-317088AE8511}" done="0">
     <text xml:space="preserve">For images containing weapons, the correct answer was "search."
 For images without weapons, the correct answer was "clear."
 </text>
   </threadedComment>
-  <threadedComment ref="D1" personId="{023F073C-A82F-2175-A266-BCA5468DB114}" id="{BDDA7502-3A80-867F-52C6-CFD5A5BB9CFD}" done="0">
+  <threadedComment ref="D1" personId="{6CBFD0F5-E47F-8D54-1A2F-22C85849A140}" id="{BDDA7502-3A80-867F-52C6-CFD5A5BB9CFD}" done="0">
     <text xml:space="preserve">Classical test theory index of difficulty (the inverse of the percent who answered correctly).
 </text>
   </threadedComment>

</xml_diff>